<commit_message>
[v1.7.0] Filas huerfanas en Resultado
</commit_message>
<xml_diff>
--- a/src/test/resources/fixtures/cierre.xlsx
+++ b/src/test/resources/fixtures/cierre.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1785,6 +1785,726 @@
         <v>9</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PROJ-20</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>reg</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>epic-r1</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>sumR1</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>u1</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>55751</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>tR1</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>99642</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>accR</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PROJ-21</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>reg</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>epic-r2</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>sumR2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>u2</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>101770</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>tR2</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>90014</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>accR</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PROJ-22</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>reg</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>epic-r2</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>sumR3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>u2</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>101770</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>tR3</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>90014</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>accR</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PROJ-23</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>HE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>reg</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>epic-r3</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>sumR4</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>u3</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>138074</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>tR4</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>99641</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>accR</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PROJ-24</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>HE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>reg</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>epic-r3</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>sumR5</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>u3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>138074</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>tR5</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>99641</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Sup</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>accR</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PROJ-30</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>huerf</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>epic-h1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>sumH1</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>u4</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>TICKETS</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>tH1</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>accH</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PROJ-31</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>huerf</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>epic-h1</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>sumH2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>u4</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>TICKETS</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>tH2</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>accH</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PROJ-32</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>huerf</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>epic-h2</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>sumH3</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>u5</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>tH3</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>90014</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>accH</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PROJ-33</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>huerf</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>epic-h3</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>sumH4</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>u1</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>P-001</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>tH4</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>MAT-HUERFANO</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>accH</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[v1.8.1] Fix resumen Responsables
</commit_message>
<xml_diff>
--- a/src/test/resources/fixtures/cierre.xlsx
+++ b/src/test/resources/fixtures/cierre.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2193,27 +2193,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PROJ-30</t>
+          <t>PROJ-25</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PF</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>huerf</t>
+          <t>pad</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>epic-h1</t>
+          <t>epic-pad</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>sumH1</t>
+          <t>sumR6</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>u4</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2238,17 +2238,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>TICKETS</t>
+          <t>P-016</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>tH1</t>
+          <t>tR6</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>M-1010</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>accH</t>
+          <t>accR</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PROJ-31</t>
+          <t>PROJ-30</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>sumH2</t>
+          <t>sumH1</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>tH2</t>
+          <t>tH1</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2353,12 +2353,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PROJ-32</t>
+          <t>PROJ-31</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2368,12 +2368,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>epic-h2</t>
+          <t>epic-h1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>sumH3</t>
+          <t>sumH2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2388,27 +2388,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>u5</t>
+          <t>u4</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>VACACIONES</t>
+          <t>TICKETS</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>tH3</t>
+          <t>tH2</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>90014</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2422,7 +2422,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -2433,75 +2433,155 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>PROJ-32</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>huerf</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>epic-h2</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>sumH3</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>u5</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>VACACIONES</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>tH3</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>90014</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>accH</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PROJ</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>PROJ-33</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>DF</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>huerf</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>epic-h3</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>sumH4</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>desc</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>u1</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>2026-02-13</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>P-001</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>tH4</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>MAT-HUERFANO</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>accH</t>
         </is>
       </c>
-      <c r="P27" t="n">
+      <c r="P28" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>